<commit_message>
Fix NAV class matching for multi-class funds
_class_suffix() replaced with _class_hint() — passes full CSV fund name
as class filter instead of single-letter suffix.

Fixes KT-INDIA-D returning KT-INDIA-A NAV (18.3199) instead of
correct D-class NAV (11.3771). Root cause: SEC API class_abbr_name
is full name 'KT-INDIA-D' not 'D', so suffix match 'D'=='KT-INDIA-D'
always failed → fell back to first item (wrong class).

Now matches via class_abbr_name.strip().upper() == csv_name.upper().
Applies to all MANUAL_SEC_NAME funds: UCHINA, UEMIF-N, KKP NDQ100-UH-E,
KKP US500-UH-E, KT-INDIA-D.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/portfolio_model.xlsx
+++ b/portfolio_model.xlsx
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -660,7 +660,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-17 17:39</t>
+          <t>Generated: 2026-05-17 17:46</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>104610</v>
+        <v>104143.76</v>
       </c>
       <c r="C6" s="5" t="n">
         <v>99600.03999999999</v>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>177334</v>
+        <v>176867.76</v>
       </c>
       <c r="C7" s="5" t="n">
         <v>173528.14</v>
@@ -764,21 +764,28 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
+          <t>🟠 STOP LOSS NEAR: KT-INDIA-D: -19.0% (SL: -20%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
           <t>🟠 CONCENTRATION BREACH: UCHINA: 24.0% &gt; 15.0% cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>🟡 ALLOCATION DRIFT: Core Growth: Underweight 15.0%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>🟡 ALLOCATION DRIFT: Thematic: Overweight 12.5%</t>
+          <t>🟡 ALLOCATION DRIFT: Core Growth: Underweight 14.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>🟡 ALLOCATION DRIFT: Thematic: Overweight 12.3%</t>
         </is>
       </c>
     </row>
@@ -1178,10 +1185,10 @@
         <v>13.6447</v>
       </c>
       <c r="D4" s="10" t="n">
-        <v>13.4469</v>
+        <v>13.443</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>9855.040000000001</v>
+        <v>9852.18</v>
       </c>
       <c r="F4" s="12">
         <f>(D4-C4)/C4</f>
@@ -1374,10 +1381,10 @@
         <v>14.5964</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>17.3264</v>
+        <v>17.415</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>2374.07</v>
+        <v>2386.21</v>
       </c>
       <c r="F11" s="11">
         <f>(D11-C11)/C11</f>
@@ -1402,10 +1409,10 @@
         <v>11.6222</v>
       </c>
       <c r="D12" s="10" t="n">
-        <v>12.8965</v>
+        <v>13.0047</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>2219.28</v>
+        <v>2237.9</v>
       </c>
       <c r="F12" s="11">
         <f>(D12-C12)/C12</f>
@@ -1430,12 +1437,12 @@
         <v>14.0501</v>
       </c>
       <c r="D13" s="10" t="n">
-        <v>18.3199</v>
+        <v>11.3771</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>1303.9</v>
-      </c>
-      <c r="F13" s="11">
+        <v>809.75</v>
+      </c>
+      <c r="F13" s="12">
         <f>(D13-C13)/C13</f>
         <v/>
       </c>
@@ -1508,7 +1515,7 @@
         <v>0.4</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>0.25</v>
+        <v>0.251</v>
       </c>
       <c r="D2" s="17">
         <f>C2-B2</f>
@@ -1525,7 +1532,7 @@
         <v>0.3</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>0.425</v>
+        <v>0.423</v>
       </c>
       <c r="D3" s="18">
         <f>C3-B3</f>
@@ -1542,7 +1549,7 @@
         <v>0.15</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>0.159</v>
+        <v>0.16</v>
       </c>
       <c r="D4" s="19">
         <f>C4-B4</f>
@@ -1621,7 +1628,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>104610</v>
+        <v>104143.76</v>
       </c>
     </row>
     <row r="6">
@@ -1631,7 +1638,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>177334</v>
+        <v>176867.76</v>
       </c>
     </row>
     <row r="7">
@@ -1651,7 +1658,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>197334</v>
+        <v>196867.76</v>
       </c>
     </row>
     <row r="10">

</xml_diff>